<commit_message>
feat(projects): per-part quality, progress dashboard, shipping UI, and mobile project screens
Backend:
- Project quality (controller/service + node-quality DTO) and per-part GLB util
- Progress dashboard service (project-progress.service + pure progress-math)
- Project model + stage services/controllers; status roll-up enhancements
- Quality-data and NCR entities/DTOs linked to assembly nodes
- Shipping service/controller updates; processes decoupled from product
- Migrations: AddProjectProcess, AddQualityFabricationLinks, DropProcessProduct

Frontend:
- Project detail expansion; new progress, shipping, and edit-dialog components
- shipping.service; routes and process form updates

Mobile:
- Project list/detail, assembly detail, and part viewer screens + projects.service
- AR part extractor and remote-model refinements; NCR create + nav/permissions

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PCS-Pricing-Model.xlsx
+++ b/PCS-Pricing-Model.xlsx
@@ -8,9 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Assumptions" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="ARR Model" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Unit Economics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="US Assumptions" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="US ARR Model" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="US Unit Economics" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="India Assumptions" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="India ARR Model" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="India Unit Economics" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -19,14 +22,15 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
-    <numFmt numFmtId="164" formatCode="0.0%"/>
-    <numFmt numFmtId="165" formatCode="0.0&quot;x&quot;"/>
-    <numFmt numFmtId="166" formatCode="$#,##0"/>
+  <numFmts count="6">
+    <numFmt numFmtId="164" formatCode="$#,##0"/>
+    <numFmt numFmtId="165" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.0&quot;x&quot;"/>
     <numFmt numFmtId="167" formatCode="0.0&quot; mo&quot;"/>
     <numFmt numFmtId="168" formatCode="0.0"/>
+    <numFmt numFmtId="169" formatCode="&quot;₹&quot;#,##0"/>
   </numFmts>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -50,6 +54,10 @@
     <font>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <color rgb="007F7F7F"/>
     </font>
   </fonts>
   <fills count="5">
@@ -101,14 +109,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -117,27 +125,33 @@
     <xf numFmtId="1" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="166" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="3" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="168" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="169" fontId="0" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="169" fontId="3" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -503,10 +517,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="112" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -522,104 +536,159 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HOW TO USE</t>
+          <t>TABS</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Edit only the BLUE cells on the 'Assumptions' tab. Everything else is a formula.</t>
+          <t xml:space="preserve">  • US Assumptions / US ARR Model / US Unit Economics  — North-American pricing in USD</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • 'ARR Model' rolls each segment's bookings forward by NRR and sums Low/Base/High scenarios.</t>
+          <t xml:space="preserve">  • India Assumptions / India ARR Model / India Unit Economics  — India pricing in INR (ex-GST)</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • 'Unit Economics' derives gross margin, CAC payback and LTV:CAC, with CAD-conversion compute broken out as COGS.</t>
-        </is>
-      </c>
+      <c r="A6" t="inlineStr"/>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>HOW TO USE</t>
+        </is>
+      </c>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>MODEL LOGIC</t>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Edit only the BLUE cells on an Assumptions tab. Everything else is a formula.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Metric = price per production SITE; floor/operator access is unlimited, only office/admin seats are counted.</t>
+          <t xml:space="preserve">  • ARR rolls each segment's bookings forward by NRR and sums Low/Base/High scenarios.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Ending ARR(t) = Ending ARR(t-1) × NRR + new-logo ARR(t), tracked per segment then summed.</t>
+          <t xml:space="preserve">  • Unit Economics derives gross margin, CAC payback and LTV:CAC; CAD-conversion compute is broken out as COGS.</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Scenarios scale the Base new-logo plan by the multipliers (Low 0.6× / Base 1.0× / High 1.5×).</t>
-        </is>
-      </c>
+      <c r="A11" t="inlineStr"/>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • LTV = annual gross profit ÷ logo churn (no expansion credit — conservative).</t>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>MODEL LOGIC</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • Net CAC = CAC − onboarding gross profit (onboarding fees substantially offset acquisition cost).</t>
+          <t xml:space="preserve">  • Metric = price per production SITE; floor/operator access unlimited, only office/admin seats counted.</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr"/>
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Ending ARR(t) = Ending ARR(t-1) × NRR + new-logo ARR(t), per segment then summed.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>CAVEATS</t>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • LTV = annual gross profit ÷ logo churn (no expansion credit — conservative).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t xml:space="preserve">  • Net CAC = CAC − onboarding gross profit (onboarding fees offset acquisition cost).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>INDIA NOTES</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Prices are ex-GST (add 18% GST; B2B customers reclaim it). Customers may deduct ~2% TDS on services.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Hosting &amp; CAD-conversion compute are USD-priced (cloud is global) so they DON'T localise down —</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    this compresses margin on the Digital Twin tier. Support/CS does localise down.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • India SMB excludes CAD compute COGS (SMB buys non-3D tiers); Mid = Digital Twin tier, so CAD applies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>CAVEATS</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
           <t xml:space="preserve">  • Figures are planning anchors, NOT committed list prices. Validate willingness-to-pay first.</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
+    <row r="26">
+      <c r="A26" t="inlineStr">
         <is>
           <t xml:space="preserve">  • LTV:CAC ratios are gated by the churn assumptions — stress-test churn before trusting them.</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • See PRICING.md for the narrative one-pager this model backs.</t>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • See PRICING.md for the narrative one-pager and the per-tier feature matrix this model backs.</t>
         </is>
       </c>
     </row>
@@ -638,15 +707,15 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Model Assumptions — edit the blue cells</t>
+          <t>Model Assumptions (USD) — edit the blue cells</t>
         </is>
       </c>
     </row>
@@ -754,7 +823,7 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>SMB net revenue retention (NRR)</t>
+          <t>SMB net revenue retention</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
@@ -934,7 +1003,7 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Hosting &amp; infra</t>
+          <t>Hosting &amp; infra (USD-priced)</t>
         </is>
       </c>
       <c r="B36" s="3" t="n">
@@ -944,7 +1013,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>CAD-conversion compute</t>
+          <t>CAD-conversion compute (USD-priced)</t>
         </is>
       </c>
       <c r="B37" s="3" t="n">
@@ -1013,22 +1082,22 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>ARR Model — ending ARR by scenario</t>
+          <t>ARR Model — ending ARR by scenario (US)</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>ENDING ARR BY SCENARIO ($)</t>
+          <t>ENDING ARR BY SCENARIO</t>
         </is>
       </c>
     </row>
@@ -1158,15 +1227,15 @@
         </is>
       </c>
       <c r="B14" s="11">
-        <f>ROUND(Assumptions!B23*Assumptions!$B$28,0)</f>
+        <f>ROUND('US Assumptions'!B23*'US Assumptions'!$B$28,0)</f>
         <v/>
       </c>
       <c r="C14" s="11">
-        <f>ROUND(Assumptions!C23*Assumptions!$B$28,0)</f>
+        <f>ROUND('US Assumptions'!C23*'US Assumptions'!$B$28,0)</f>
         <v/>
       </c>
       <c r="D14" s="11">
-        <f>ROUND(Assumptions!D23*Assumptions!$B$28,0)</f>
+        <f>ROUND('US Assumptions'!D23*'US Assumptions'!$B$28,0)</f>
         <v/>
       </c>
     </row>
@@ -1177,15 +1246,15 @@
         </is>
       </c>
       <c r="B15" s="11">
-        <f>ROUND(Assumptions!B24*Assumptions!$B$28,0)</f>
+        <f>ROUND('US Assumptions'!B24*'US Assumptions'!$B$28,0)</f>
         <v/>
       </c>
       <c r="C15" s="11">
-        <f>ROUND(Assumptions!C24*Assumptions!$B$28,0)</f>
+        <f>ROUND('US Assumptions'!C24*'US Assumptions'!$B$28,0)</f>
         <v/>
       </c>
       <c r="D15" s="11">
-        <f>ROUND(Assumptions!D24*Assumptions!$B$28,0)</f>
+        <f>ROUND('US Assumptions'!D24*'US Assumptions'!$B$28,0)</f>
         <v/>
       </c>
     </row>
@@ -1196,15 +1265,15 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>B14*Assumptions!$B$10</f>
+        <f>B14*'US Assumptions'!$B$10</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>C14*Assumptions!$B$10</f>
+        <f>C14*'US Assumptions'!$B$10</f>
         <v/>
       </c>
       <c r="D16" s="12">
-        <f>D14*Assumptions!$B$10</f>
+        <f>D14*'US Assumptions'!$B$10</f>
         <v/>
       </c>
     </row>
@@ -1215,15 +1284,15 @@
         </is>
       </c>
       <c r="B17" s="12">
-        <f>B15*Assumptions!$B$11</f>
+        <f>B15*'US Assumptions'!$B$11</f>
         <v/>
       </c>
       <c r="C17" s="12">
-        <f>C15*Assumptions!$B$11</f>
+        <f>C15*'US Assumptions'!$B$11</f>
         <v/>
       </c>
       <c r="D17" s="12">
-        <f>D15*Assumptions!$B$11</f>
+        <f>D15*'US Assumptions'!$B$11</f>
         <v/>
       </c>
     </row>
@@ -1238,11 +1307,11 @@
         <v/>
       </c>
       <c r="C18" s="12">
-        <f>B18*Assumptions!$B$16+C16</f>
+        <f>B18*'US Assumptions'!$B$16+C16</f>
         <v/>
       </c>
       <c r="D18" s="12">
-        <f>C18*Assumptions!$B$16+D16</f>
+        <f>C18*'US Assumptions'!$B$16+D16</f>
         <v/>
       </c>
     </row>
@@ -1257,11 +1326,11 @@
         <v/>
       </c>
       <c r="C19" s="12">
-        <f>B19*Assumptions!$B$17+C17</f>
+        <f>B19*'US Assumptions'!$B$17+C17</f>
         <v/>
       </c>
       <c r="D19" s="12">
-        <f>C19*Assumptions!$B$17+D17</f>
+        <f>C19*'US Assumptions'!$B$17+D17</f>
         <v/>
       </c>
     </row>
@@ -1291,15 +1360,15 @@
         </is>
       </c>
       <c r="B21" s="12">
-        <f>B14*Assumptions!$B$12+B15*Assumptions!$B$13</f>
+        <f>B14*'US Assumptions'!$B$12+B15*'US Assumptions'!$B$13</f>
         <v/>
       </c>
       <c r="C21" s="12">
-        <f>C14*Assumptions!$B$12+C15*Assumptions!$B$13</f>
+        <f>C14*'US Assumptions'!$B$12+C15*'US Assumptions'!$B$13</f>
         <v/>
       </c>
       <c r="D21" s="12">
-        <f>D14*Assumptions!$B$12+D15*Assumptions!$B$13</f>
+        <f>D14*'US Assumptions'!$B$12+D15*'US Assumptions'!$B$13</f>
         <v/>
       </c>
     </row>
@@ -1335,15 +1404,15 @@
         </is>
       </c>
       <c r="B26" s="11">
-        <f>ROUND(Assumptions!B23*Assumptions!$C$28,0)</f>
+        <f>ROUND('US Assumptions'!B23*'US Assumptions'!$C$28,0)</f>
         <v/>
       </c>
       <c r="C26" s="11">
-        <f>ROUND(Assumptions!C23*Assumptions!$C$28,0)</f>
+        <f>ROUND('US Assumptions'!C23*'US Assumptions'!$C$28,0)</f>
         <v/>
       </c>
       <c r="D26" s="11">
-        <f>ROUND(Assumptions!D23*Assumptions!$C$28,0)</f>
+        <f>ROUND('US Assumptions'!D23*'US Assumptions'!$C$28,0)</f>
         <v/>
       </c>
     </row>
@@ -1354,15 +1423,15 @@
         </is>
       </c>
       <c r="B27" s="11">
-        <f>ROUND(Assumptions!B24*Assumptions!$C$28,0)</f>
+        <f>ROUND('US Assumptions'!B24*'US Assumptions'!$C$28,0)</f>
         <v/>
       </c>
       <c r="C27" s="11">
-        <f>ROUND(Assumptions!C24*Assumptions!$C$28,0)</f>
+        <f>ROUND('US Assumptions'!C24*'US Assumptions'!$C$28,0)</f>
         <v/>
       </c>
       <c r="D27" s="11">
-        <f>ROUND(Assumptions!D24*Assumptions!$C$28,0)</f>
+        <f>ROUND('US Assumptions'!D24*'US Assumptions'!$C$28,0)</f>
         <v/>
       </c>
     </row>
@@ -1373,15 +1442,15 @@
         </is>
       </c>
       <c r="B28" s="12">
-        <f>B26*Assumptions!$B$10</f>
+        <f>B26*'US Assumptions'!$B$10</f>
         <v/>
       </c>
       <c r="C28" s="12">
-        <f>C26*Assumptions!$B$10</f>
+        <f>C26*'US Assumptions'!$B$10</f>
         <v/>
       </c>
       <c r="D28" s="12">
-        <f>D26*Assumptions!$B$10</f>
+        <f>D26*'US Assumptions'!$B$10</f>
         <v/>
       </c>
     </row>
@@ -1392,15 +1461,15 @@
         </is>
       </c>
       <c r="B29" s="12">
-        <f>B27*Assumptions!$B$11</f>
+        <f>B27*'US Assumptions'!$B$11</f>
         <v/>
       </c>
       <c r="C29" s="12">
-        <f>C27*Assumptions!$B$11</f>
+        <f>C27*'US Assumptions'!$B$11</f>
         <v/>
       </c>
       <c r="D29" s="12">
-        <f>D27*Assumptions!$B$11</f>
+        <f>D27*'US Assumptions'!$B$11</f>
         <v/>
       </c>
     </row>
@@ -1415,11 +1484,11 @@
         <v/>
       </c>
       <c r="C30" s="12">
-        <f>B30*Assumptions!$B$16+C28</f>
+        <f>B30*'US Assumptions'!$B$16+C28</f>
         <v/>
       </c>
       <c r="D30" s="12">
-        <f>C30*Assumptions!$B$16+D28</f>
+        <f>C30*'US Assumptions'!$B$16+D28</f>
         <v/>
       </c>
     </row>
@@ -1434,11 +1503,11 @@
         <v/>
       </c>
       <c r="C31" s="12">
-        <f>B31*Assumptions!$B$17+C29</f>
+        <f>B31*'US Assumptions'!$B$17+C29</f>
         <v/>
       </c>
       <c r="D31" s="12">
-        <f>C31*Assumptions!$B$17+D29</f>
+        <f>C31*'US Assumptions'!$B$17+D29</f>
         <v/>
       </c>
     </row>
@@ -1468,15 +1537,15 @@
         </is>
       </c>
       <c r="B33" s="12">
-        <f>B26*Assumptions!$B$12+B27*Assumptions!$B$13</f>
+        <f>B26*'US Assumptions'!$B$12+B27*'US Assumptions'!$B$13</f>
         <v/>
       </c>
       <c r="C33" s="12">
-        <f>C26*Assumptions!$B$12+C27*Assumptions!$B$13</f>
+        <f>C26*'US Assumptions'!$B$12+C27*'US Assumptions'!$B$13</f>
         <v/>
       </c>
       <c r="D33" s="12">
-        <f>D26*Assumptions!$B$12+D27*Assumptions!$B$13</f>
+        <f>D26*'US Assumptions'!$B$12+D27*'US Assumptions'!$B$13</f>
         <v/>
       </c>
     </row>
@@ -1512,15 +1581,15 @@
         </is>
       </c>
       <c r="B38" s="11">
-        <f>ROUND(Assumptions!B23*Assumptions!$D$28,0)</f>
+        <f>ROUND('US Assumptions'!B23*'US Assumptions'!$D$28,0)</f>
         <v/>
       </c>
       <c r="C38" s="11">
-        <f>ROUND(Assumptions!C23*Assumptions!$D$28,0)</f>
+        <f>ROUND('US Assumptions'!C23*'US Assumptions'!$D$28,0)</f>
         <v/>
       </c>
       <c r="D38" s="11">
-        <f>ROUND(Assumptions!D23*Assumptions!$D$28,0)</f>
+        <f>ROUND('US Assumptions'!D23*'US Assumptions'!$D$28,0)</f>
         <v/>
       </c>
     </row>
@@ -1531,15 +1600,15 @@
         </is>
       </c>
       <c r="B39" s="11">
-        <f>ROUND(Assumptions!B24*Assumptions!$D$28,0)</f>
+        <f>ROUND('US Assumptions'!B24*'US Assumptions'!$D$28,0)</f>
         <v/>
       </c>
       <c r="C39" s="11">
-        <f>ROUND(Assumptions!C24*Assumptions!$D$28,0)</f>
+        <f>ROUND('US Assumptions'!C24*'US Assumptions'!$D$28,0)</f>
         <v/>
       </c>
       <c r="D39" s="11">
-        <f>ROUND(Assumptions!D24*Assumptions!$D$28,0)</f>
+        <f>ROUND('US Assumptions'!D24*'US Assumptions'!$D$28,0)</f>
         <v/>
       </c>
     </row>
@@ -1550,15 +1619,15 @@
         </is>
       </c>
       <c r="B40" s="12">
-        <f>B38*Assumptions!$B$10</f>
+        <f>B38*'US Assumptions'!$B$10</f>
         <v/>
       </c>
       <c r="C40" s="12">
-        <f>C38*Assumptions!$B$10</f>
+        <f>C38*'US Assumptions'!$B$10</f>
         <v/>
       </c>
       <c r="D40" s="12">
-        <f>D38*Assumptions!$B$10</f>
+        <f>D38*'US Assumptions'!$B$10</f>
         <v/>
       </c>
     </row>
@@ -1569,15 +1638,15 @@
         </is>
       </c>
       <c r="B41" s="12">
-        <f>B39*Assumptions!$B$11</f>
+        <f>B39*'US Assumptions'!$B$11</f>
         <v/>
       </c>
       <c r="C41" s="12">
-        <f>C39*Assumptions!$B$11</f>
+        <f>C39*'US Assumptions'!$B$11</f>
         <v/>
       </c>
       <c r="D41" s="12">
-        <f>D39*Assumptions!$B$11</f>
+        <f>D39*'US Assumptions'!$B$11</f>
         <v/>
       </c>
     </row>
@@ -1592,11 +1661,11 @@
         <v/>
       </c>
       <c r="C42" s="12">
-        <f>B42*Assumptions!$B$16+C40</f>
+        <f>B42*'US Assumptions'!$B$16+C40</f>
         <v/>
       </c>
       <c r="D42" s="12">
-        <f>C42*Assumptions!$B$16+D40</f>
+        <f>C42*'US Assumptions'!$B$16+D40</f>
         <v/>
       </c>
     </row>
@@ -1611,11 +1680,11 @@
         <v/>
       </c>
       <c r="C43" s="12">
-        <f>B43*Assumptions!$B$17+C41</f>
+        <f>B43*'US Assumptions'!$B$17+C41</f>
         <v/>
       </c>
       <c r="D43" s="12">
-        <f>C43*Assumptions!$B$17+D41</f>
+        <f>C43*'US Assumptions'!$B$17+D41</f>
         <v/>
       </c>
     </row>
@@ -1645,15 +1714,15 @@
         </is>
       </c>
       <c r="B45" s="12">
-        <f>B38*Assumptions!$B$12+B39*Assumptions!$B$13</f>
+        <f>B38*'US Assumptions'!$B$12+B39*'US Assumptions'!$B$13</f>
         <v/>
       </c>
       <c r="C45" s="12">
-        <f>C38*Assumptions!$B$12+C39*Assumptions!$B$13</f>
+        <f>C38*'US Assumptions'!$B$12+C39*'US Assumptions'!$B$13</f>
         <v/>
       </c>
       <c r="D45" s="12">
-        <f>D38*Assumptions!$B$12+D39*Assumptions!$B$13</f>
+        <f>D38*'US Assumptions'!$B$12+D39*'US Assumptions'!$B$13</f>
         <v/>
       </c>
     </row>
@@ -1671,10 +1740,10 @@
   <dimension ref="A1:F27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="28" customWidth="1" min="1" max="1"/>
-    <col width="13" customWidth="1" min="2" max="2"/>
-    <col width="13" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
     <col width="18" customWidth="1" min="5" max="5"/>
     <col width="8" customWidth="1" min="6" max="6"/>
   </cols>
@@ -1682,7 +1751,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Unit Economics</t>
+          <t>Unit Economics (US)</t>
         </is>
       </c>
     </row>
@@ -1721,15 +1790,15 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ACV ($/yr)</t>
-        </is>
-      </c>
-      <c r="B4" s="15">
-        <f>Assumptions!B10</f>
-        <v/>
-      </c>
-      <c r="C4" s="15">
-        <f>Assumptions!B11</f>
+          <t>ACV / yr</t>
+        </is>
+      </c>
+      <c r="B4" s="12">
+        <f>'US Assumptions'!B10</f>
+        <v/>
+      </c>
+      <c r="C4" s="12">
+        <f>'US Assumptions'!B11</f>
         <v/>
       </c>
       <c r="D4" s="10">
@@ -1741,8 +1810,8 @@
           <t>SMB logos (Base)</t>
         </is>
       </c>
-      <c r="F4" s="16">
-        <f>SUM(Assumptions!B23:D23)</f>
+      <c r="F4" s="15">
+        <f>SUM('US Assumptions'!B23:D23)</f>
         <v/>
       </c>
     </row>
@@ -1753,11 +1822,11 @@
         </is>
       </c>
       <c r="B5" s="11">
-        <f>Assumptions!B42</f>
+        <f>'US Assumptions'!B42</f>
         <v/>
       </c>
       <c r="C5" s="11">
-        <f>Assumptions!B43</f>
+        <f>'US Assumptions'!B43</f>
         <v/>
       </c>
       <c r="E5" t="inlineStr">
@@ -1765,8 +1834,8 @@
           <t>Mid logos (Base)</t>
         </is>
       </c>
-      <c r="F5" s="16">
-        <f>SUM(Assumptions!B24:D24)</f>
+      <c r="F5" s="15">
+        <f>SUM('US Assumptions'!B24:D24)</f>
         <v/>
       </c>
     </row>
@@ -1777,11 +1846,11 @@
         </is>
       </c>
       <c r="B6" s="12">
-        <f>B5*Assumptions!$B$36</f>
+        <f>B5*'US Assumptions'!$B$36</f>
         <v/>
       </c>
       <c r="C6" s="12">
-        <f>C5*Assumptions!$B$36</f>
+        <f>C5*'US Assumptions'!$B$36</f>
         <v/>
       </c>
     </row>
@@ -1792,11 +1861,11 @@
         </is>
       </c>
       <c r="B7" s="12">
-        <f>B5*Assumptions!$B$37</f>
+        <f>B5*'US Assumptions'!$B$37</f>
         <v/>
       </c>
       <c r="C7" s="12">
-        <f>C5*Assumptions!$B$37</f>
+        <f>C5*'US Assumptions'!$B$37</f>
         <v/>
       </c>
     </row>
@@ -1807,11 +1876,11 @@
         </is>
       </c>
       <c r="B8" s="12">
-        <f>B5*Assumptions!$B$38</f>
+        <f>B5*'US Assumptions'!$B$38</f>
         <v/>
       </c>
       <c r="C8" s="12">
-        <f>C5*Assumptions!$B$38</f>
+        <f>C5*'US Assumptions'!$B$38</f>
         <v/>
       </c>
     </row>
@@ -1822,11 +1891,11 @@
         </is>
       </c>
       <c r="B9" s="12">
-        <f>B4*Assumptions!$B$39</f>
+        <f>B4*'US Assumptions'!$B$39</f>
         <v/>
       </c>
       <c r="C9" s="12">
-        <f>C4*Assumptions!$B$39</f>
+        <f>C4*'US Assumptions'!$B$39</f>
         <v/>
       </c>
     </row>
@@ -1836,11 +1905,11 @@
           <t>Total COGS</t>
         </is>
       </c>
-      <c r="B10" s="15">
+      <c r="B10" s="12">
         <f>SUM(B6:B9)</f>
         <v/>
       </c>
-      <c r="C10" s="15">
+      <c r="C10" s="12">
         <f>SUM(C6:C9)</f>
         <v/>
       </c>
@@ -1852,14 +1921,14 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Gross profit ($/yr)</t>
-        </is>
-      </c>
-      <c r="B11" s="15">
+          <t>Gross profit / yr</t>
+        </is>
+      </c>
+      <c r="B11" s="12">
         <f>B4-B10</f>
         <v/>
       </c>
-      <c r="C11" s="15">
+      <c r="C11" s="12">
         <f>C4-C10</f>
         <v/>
       </c>
@@ -1874,15 +1943,15 @@
           <t>Gross margin %</t>
         </is>
       </c>
-      <c r="B12" s="17">
+      <c r="B12" s="16">
         <f>B11/B4</f>
         <v/>
       </c>
-      <c r="C12" s="17">
+      <c r="C12" s="16">
         <f>C11/C4</f>
         <v/>
       </c>
-      <c r="D12" s="18">
+      <c r="D12" s="17">
         <f>D11/D4</f>
         <v/>
       </c>
@@ -1893,12 +1962,12 @@
           <t>CAC per logo</t>
         </is>
       </c>
-      <c r="B14" s="15">
-        <f>Assumptions!B31</f>
-        <v/>
-      </c>
-      <c r="C14" s="15">
-        <f>Assumptions!B32</f>
+      <c r="B14" s="12">
+        <f>'US Assumptions'!B31</f>
+        <v/>
+      </c>
+      <c r="C14" s="12">
+        <f>'US Assumptions'!B32</f>
         <v/>
       </c>
       <c r="D14" s="10">
@@ -1912,12 +1981,12 @@
           <t>Onboarding fee</t>
         </is>
       </c>
-      <c r="B15" s="15">
-        <f>Assumptions!B12</f>
-        <v/>
-      </c>
-      <c r="C15" s="15">
-        <f>Assumptions!B13</f>
+      <c r="B15" s="12">
+        <f>'US Assumptions'!B12</f>
+        <v/>
+      </c>
+      <c r="C15" s="12">
+        <f>'US Assumptions'!B13</f>
         <v/>
       </c>
     </row>
@@ -1928,11 +1997,11 @@
         </is>
       </c>
       <c r="B16" s="12">
-        <f>B15*Assumptions!$B$33</f>
+        <f>B15*'US Assumptions'!$B$33</f>
         <v/>
       </c>
       <c r="C16" s="12">
-        <f>C15*Assumptions!$B$33</f>
+        <f>C15*'US Assumptions'!$B$33</f>
         <v/>
       </c>
     </row>
@@ -1942,11 +2011,11 @@
           <t>Net CAC (CAC − onb. GP)</t>
         </is>
       </c>
-      <c r="B17" s="15">
+      <c r="B17" s="12">
         <f>B14-B16</f>
         <v/>
       </c>
-      <c r="C17" s="15">
+      <c r="C17" s="12">
         <f>C14-C16</f>
         <v/>
       </c>
@@ -1976,15 +2045,15 @@
           <t>CAC payback (gross)</t>
         </is>
       </c>
-      <c r="B20" s="19">
+      <c r="B20" s="18">
         <f>B14/B19</f>
         <v/>
       </c>
-      <c r="C20" s="19">
+      <c r="C20" s="18">
         <f>C14/C19</f>
         <v/>
       </c>
-      <c r="D20" s="20">
+      <c r="D20" s="19">
         <f>D14/(D11/12)</f>
         <v/>
       </c>
@@ -1995,15 +2064,15 @@
           <t>Net CAC payback</t>
         </is>
       </c>
-      <c r="B21" s="19">
+      <c r="B21" s="18">
         <f>B17/B19</f>
         <v/>
       </c>
-      <c r="C21" s="19">
+      <c r="C21" s="18">
         <f>C17/C19</f>
         <v/>
       </c>
-      <c r="D21" s="20">
+      <c r="D21" s="19">
         <f>D17/(D11/12)</f>
         <v/>
       </c>
@@ -2014,12 +2083,12 @@
           <t>Logo churn / yr</t>
         </is>
       </c>
-      <c r="B23" s="17">
-        <f>Assumptions!B18</f>
-        <v/>
-      </c>
-      <c r="C23" s="17">
-        <f>Assumptions!B19</f>
+      <c r="B23" s="16">
+        <f>'US Assumptions'!B18</f>
+        <v/>
+      </c>
+      <c r="C23" s="16">
+        <f>'US Assumptions'!B19</f>
         <v/>
       </c>
     </row>
@@ -2029,11 +2098,11 @@
           <t>Customer lifetime (yrs)</t>
         </is>
       </c>
-      <c r="B24" s="21">
+      <c r="B24" s="20">
         <f>1/B23</f>
         <v/>
       </c>
-      <c r="C24" s="21">
+      <c r="C24" s="20">
         <f>1/C23</f>
         <v/>
       </c>
@@ -2044,11 +2113,11 @@
           <t>LTV (gross margin)</t>
         </is>
       </c>
-      <c r="B25" s="15">
+      <c r="B25" s="12">
         <f>B11*B24</f>
         <v/>
       </c>
-      <c r="C25" s="15">
+      <c r="C25" s="12">
         <f>C11*C24</f>
         <v/>
       </c>
@@ -2063,15 +2132,15 @@
           <t>LTV:CAC (gross)</t>
         </is>
       </c>
-      <c r="B26" s="22">
+      <c r="B26" s="21">
         <f>B25/B14</f>
         <v/>
       </c>
-      <c r="C26" s="22">
+      <c r="C26" s="21">
         <f>C25/C14</f>
         <v/>
       </c>
-      <c r="D26" s="23">
+      <c r="D26" s="22">
         <f>D25/D14</f>
         <v/>
       </c>
@@ -2082,17 +2151,1496 @@
           <t>LTV:CAC (net CAC)</t>
         </is>
       </c>
-      <c r="B27" s="22">
+      <c r="B27" s="21">
         <f>B25/B17</f>
         <v/>
       </c>
-      <c r="C27" s="22">
+      <c r="C27" s="21">
         <f>C25/C17</f>
         <v/>
       </c>
-      <c r="D27" s="23">
+      <c r="D27" s="22">
         <f>D25/D17</f>
         <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Model Assumptions (INR, ex-GST) — edit the blue cells</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>PRICING (per site / year)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Core MES</t>
+        </is>
+      </c>
+      <c r="B4" s="23" t="n">
+        <v>144000</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Quality &amp; Traceability</t>
+        </is>
+      </c>
+      <c r="B5" s="23" t="n">
+        <v>360000</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Digital Twin / AR</t>
+        </is>
+      </c>
+      <c r="B6" s="23" t="n">
+        <v>600000</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Office/admin seat / yr</t>
+        </is>
+      </c>
+      <c r="B7" s="23" t="n">
+        <v>10800</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>SEGMENT ECONOMICS</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>SMB blended ACV</t>
+        </is>
+      </c>
+      <c r="B10" s="23" t="n">
+        <v>250000</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Mid-market blended ACV</t>
+        </is>
+      </c>
+      <c r="B11" s="23" t="n">
+        <v>1750000</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>SMB onboarding (one-time)</t>
+        </is>
+      </c>
+      <c r="B12" s="23" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Mid onboarding (one-time)</t>
+        </is>
+      </c>
+      <c r="B13" s="23" t="n">
+        <v>350000</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>RETENTION</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SMB net revenue retention</t>
+        </is>
+      </c>
+      <c r="B16" s="4" t="n">
+        <v>0.95</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mid NRR</t>
+        </is>
+      </c>
+      <c r="B17" s="4" t="n">
+        <v>1.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SMB logo churn / yr</t>
+        </is>
+      </c>
+      <c r="B18" s="4" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Mid logo churn / yr</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="n">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>NEW-LOGO PLAN (Base scenario)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>SMB new logos</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="n">
+        <v>20</v>
+      </c>
+      <c r="C23" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="D23" s="6" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Mid new logos</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C24" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="D24" s="6" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>SCENARIO MULTIPLIERS</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>× Base plan</t>
+        </is>
+      </c>
+      <c r="B28" s="7" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="C28" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D28" s="7" t="n">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>UNIT ECONOMICS INPUTS</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>SMB CAC per logo</t>
+        </is>
+      </c>
+      <c r="B31" s="23" t="n">
+        <v>125000</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Mid CAC per logo</t>
+        </is>
+      </c>
+      <c r="B32" s="23" t="n">
+        <v>800000</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Onboarding gross margin %</t>
+        </is>
+      </c>
+      <c r="B33" s="4" t="n">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>COGS per SITE / year</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>Hosting &amp; infra (USD-priced)</t>
+        </is>
+      </c>
+      <c r="B36" s="23" t="n">
+        <v>35000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>CAD-conversion compute (USD-priced)</t>
+        </is>
+      </c>
+      <c r="B37" s="23" t="n">
+        <v>100000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>Support / CS</t>
+        </is>
+      </c>
+      <c r="B38" s="23" t="n">
+        <v>20000</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Payment processing (% of ACV)</t>
+        </is>
+      </c>
+      <c r="B39" s="4" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>SITES PER CUSTOMER</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SMB sites</t>
+        </is>
+      </c>
+      <c r="B42" s="6" t="n">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Mid sites</t>
+        </is>
+      </c>
+      <c r="B43" s="6" t="n">
+        <v>4</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>ARR Model — ending ARR by scenario (India)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>ENDING ARR BY SCENARIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr"/>
+      <c r="B4" s="9" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="C4" s="9" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="D4" s="9" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="B5" s="24">
+        <f>B20</f>
+        <v/>
+      </c>
+      <c r="C5" s="24">
+        <f>C20</f>
+        <v/>
+      </c>
+      <c r="D5" s="24">
+        <f>D20</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B6" s="24">
+        <f>B32</f>
+        <v/>
+      </c>
+      <c r="C6" s="24">
+        <f>C32</f>
+        <v/>
+      </c>
+      <c r="D6" s="24">
+        <f>D32</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="B7" s="24">
+        <f>B44</f>
+        <v/>
+      </c>
+      <c r="C7" s="24">
+        <f>C44</f>
+        <v/>
+      </c>
+      <c r="D7" s="24">
+        <f>D44</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>Services revenue (one-time, Base)</t>
+        </is>
+      </c>
+      <c r="B9" s="24">
+        <f>B33</f>
+        <v/>
+      </c>
+      <c r="C9" s="24">
+        <f>C33</f>
+        <v/>
+      </c>
+      <c r="D9" s="24">
+        <f>D33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>LOW SCENARIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="inlineStr"/>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>SMB new logos</t>
+        </is>
+      </c>
+      <c r="B14" s="11">
+        <f>ROUND('India Assumptions'!B23*'India Assumptions'!$B$28,0)</f>
+        <v/>
+      </c>
+      <c r="C14" s="11">
+        <f>ROUND('India Assumptions'!C23*'India Assumptions'!$B$28,0)</f>
+        <v/>
+      </c>
+      <c r="D14" s="11">
+        <f>ROUND('India Assumptions'!D23*'India Assumptions'!$B$28,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Mid new logos</t>
+        </is>
+      </c>
+      <c r="B15" s="11">
+        <f>ROUND('India Assumptions'!B24*'India Assumptions'!$B$28,0)</f>
+        <v/>
+      </c>
+      <c r="C15" s="11">
+        <f>ROUND('India Assumptions'!C24*'India Assumptions'!$B$28,0)</f>
+        <v/>
+      </c>
+      <c r="D15" s="11">
+        <f>ROUND('India Assumptions'!D24*'India Assumptions'!$B$28,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>SMB new ARR</t>
+        </is>
+      </c>
+      <c r="B16" s="25">
+        <f>B14*'India Assumptions'!$B$10</f>
+        <v/>
+      </c>
+      <c r="C16" s="25">
+        <f>C14*'India Assumptions'!$B$10</f>
+        <v/>
+      </c>
+      <c r="D16" s="25">
+        <f>D14*'India Assumptions'!$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Mid new ARR</t>
+        </is>
+      </c>
+      <c r="B17" s="25">
+        <f>B15*'India Assumptions'!$B$11</f>
+        <v/>
+      </c>
+      <c r="C17" s="25">
+        <f>C15*'India Assumptions'!$B$11</f>
+        <v/>
+      </c>
+      <c r="D17" s="25">
+        <f>D15*'India Assumptions'!$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>SMB ending ARR</t>
+        </is>
+      </c>
+      <c r="B18" s="25">
+        <f>B16</f>
+        <v/>
+      </c>
+      <c r="C18" s="25">
+        <f>B18*'India Assumptions'!$B$16+C16</f>
+        <v/>
+      </c>
+      <c r="D18" s="25">
+        <f>C18*'India Assumptions'!$B$16+D16</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Mid ending ARR</t>
+        </is>
+      </c>
+      <c r="B19" s="25">
+        <f>B17</f>
+        <v/>
+      </c>
+      <c r="C19" s="25">
+        <f>B19*'India Assumptions'!$B$17+C17</f>
+        <v/>
+      </c>
+      <c r="D19" s="25">
+        <f>C19*'India Assumptions'!$B$17+D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Total ending ARR</t>
+        </is>
+      </c>
+      <c r="B20" s="26">
+        <f>B18+B19</f>
+        <v/>
+      </c>
+      <c r="C20" s="26">
+        <f>C18+C19</f>
+        <v/>
+      </c>
+      <c r="D20" s="26">
+        <f>D18+D19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Services (one-time)</t>
+        </is>
+      </c>
+      <c r="B21" s="25">
+        <f>B14*'India Assumptions'!$B$12+B15*'India Assumptions'!$B$13</f>
+        <v/>
+      </c>
+      <c r="C21" s="25">
+        <f>C14*'India Assumptions'!$B$12+C15*'India Assumptions'!$B$13</f>
+        <v/>
+      </c>
+      <c r="D21" s="25">
+        <f>D14*'India Assumptions'!$B$12+D15*'India Assumptions'!$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>BASE SCENARIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="8" t="inlineStr"/>
+      <c r="B25" s="9" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="C25" s="9" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="D25" s="9" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>SMB new logos</t>
+        </is>
+      </c>
+      <c r="B26" s="11">
+        <f>ROUND('India Assumptions'!B23*'India Assumptions'!$C$28,0)</f>
+        <v/>
+      </c>
+      <c r="C26" s="11">
+        <f>ROUND('India Assumptions'!C23*'India Assumptions'!$C$28,0)</f>
+        <v/>
+      </c>
+      <c r="D26" s="11">
+        <f>ROUND('India Assumptions'!D23*'India Assumptions'!$C$28,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Mid new logos</t>
+        </is>
+      </c>
+      <c r="B27" s="11">
+        <f>ROUND('India Assumptions'!B24*'India Assumptions'!$C$28,0)</f>
+        <v/>
+      </c>
+      <c r="C27" s="11">
+        <f>ROUND('India Assumptions'!C24*'India Assumptions'!$C$28,0)</f>
+        <v/>
+      </c>
+      <c r="D27" s="11">
+        <f>ROUND('India Assumptions'!D24*'India Assumptions'!$C$28,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>SMB new ARR</t>
+        </is>
+      </c>
+      <c r="B28" s="25">
+        <f>B26*'India Assumptions'!$B$10</f>
+        <v/>
+      </c>
+      <c r="C28" s="25">
+        <f>C26*'India Assumptions'!$B$10</f>
+        <v/>
+      </c>
+      <c r="D28" s="25">
+        <f>D26*'India Assumptions'!$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Mid new ARR</t>
+        </is>
+      </c>
+      <c r="B29" s="25">
+        <f>B27*'India Assumptions'!$B$11</f>
+        <v/>
+      </c>
+      <c r="C29" s="25">
+        <f>C27*'India Assumptions'!$B$11</f>
+        <v/>
+      </c>
+      <c r="D29" s="25">
+        <f>D27*'India Assumptions'!$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>SMB ending ARR</t>
+        </is>
+      </c>
+      <c r="B30" s="25">
+        <f>B28</f>
+        <v/>
+      </c>
+      <c r="C30" s="25">
+        <f>B30*'India Assumptions'!$B$16+C28</f>
+        <v/>
+      </c>
+      <c r="D30" s="25">
+        <f>C30*'India Assumptions'!$B$16+D28</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Mid ending ARR</t>
+        </is>
+      </c>
+      <c r="B31" s="25">
+        <f>B29</f>
+        <v/>
+      </c>
+      <c r="C31" s="25">
+        <f>B31*'India Assumptions'!$B$17+C29</f>
+        <v/>
+      </c>
+      <c r="D31" s="25">
+        <f>C31*'India Assumptions'!$B$17+D29</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Total ending ARR</t>
+        </is>
+      </c>
+      <c r="B32" s="26">
+        <f>B30+B31</f>
+        <v/>
+      </c>
+      <c r="C32" s="26">
+        <f>C30+C31</f>
+        <v/>
+      </c>
+      <c r="D32" s="26">
+        <f>D30+D31</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Services (one-time)</t>
+        </is>
+      </c>
+      <c r="B33" s="25">
+        <f>B26*'India Assumptions'!$B$12+B27*'India Assumptions'!$B$13</f>
+        <v/>
+      </c>
+      <c r="C33" s="25">
+        <f>C26*'India Assumptions'!$B$12+C27*'India Assumptions'!$B$13</f>
+        <v/>
+      </c>
+      <c r="D33" s="25">
+        <f>D26*'India Assumptions'!$B$12+D27*'India Assumptions'!$B$13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>HIGH SCENARIO</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="8" t="inlineStr"/>
+      <c r="B37" s="9" t="inlineStr">
+        <is>
+          <t>Y1</t>
+        </is>
+      </c>
+      <c r="C37" s="9" t="inlineStr">
+        <is>
+          <t>Y2</t>
+        </is>
+      </c>
+      <c r="D37" s="9" t="inlineStr">
+        <is>
+          <t>Y3</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>SMB new logos</t>
+        </is>
+      </c>
+      <c r="B38" s="11">
+        <f>ROUND('India Assumptions'!B23*'India Assumptions'!$D$28,0)</f>
+        <v/>
+      </c>
+      <c r="C38" s="11">
+        <f>ROUND('India Assumptions'!C23*'India Assumptions'!$D$28,0)</f>
+        <v/>
+      </c>
+      <c r="D38" s="11">
+        <f>ROUND('India Assumptions'!D23*'India Assumptions'!$D$28,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>Mid new logos</t>
+        </is>
+      </c>
+      <c r="B39" s="11">
+        <f>ROUND('India Assumptions'!B24*'India Assumptions'!$D$28,0)</f>
+        <v/>
+      </c>
+      <c r="C39" s="11">
+        <f>ROUND('India Assumptions'!C24*'India Assumptions'!$D$28,0)</f>
+        <v/>
+      </c>
+      <c r="D39" s="11">
+        <f>ROUND('India Assumptions'!D24*'India Assumptions'!$D$28,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>SMB new ARR</t>
+        </is>
+      </c>
+      <c r="B40" s="25">
+        <f>B38*'India Assumptions'!$B$10</f>
+        <v/>
+      </c>
+      <c r="C40" s="25">
+        <f>C38*'India Assumptions'!$B$10</f>
+        <v/>
+      </c>
+      <c r="D40" s="25">
+        <f>D38*'India Assumptions'!$B$10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>Mid new ARR</t>
+        </is>
+      </c>
+      <c r="B41" s="25">
+        <f>B39*'India Assumptions'!$B$11</f>
+        <v/>
+      </c>
+      <c r="C41" s="25">
+        <f>C39*'India Assumptions'!$B$11</f>
+        <v/>
+      </c>
+      <c r="D41" s="25">
+        <f>D39*'India Assumptions'!$B$11</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>SMB ending ARR</t>
+        </is>
+      </c>
+      <c r="B42" s="25">
+        <f>B40</f>
+        <v/>
+      </c>
+      <c r="C42" s="25">
+        <f>B42*'India Assumptions'!$B$16+C40</f>
+        <v/>
+      </c>
+      <c r="D42" s="25">
+        <f>C42*'India Assumptions'!$B$16+D40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>Mid ending ARR</t>
+        </is>
+      </c>
+      <c r="B43" s="25">
+        <f>B41</f>
+        <v/>
+      </c>
+      <c r="C43" s="25">
+        <f>B43*'India Assumptions'!$B$17+C41</f>
+        <v/>
+      </c>
+      <c r="D43" s="25">
+        <f>C43*'India Assumptions'!$B$17+D41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>Total ending ARR</t>
+        </is>
+      </c>
+      <c r="B44" s="26">
+        <f>B42+B43</f>
+        <v/>
+      </c>
+      <c r="C44" s="26">
+        <f>C42+C43</f>
+        <v/>
+      </c>
+      <c r="D44" s="26">
+        <f>D42+D43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>Services (one-time)</t>
+        </is>
+      </c>
+      <c r="B45" s="25">
+        <f>B38*'India Assumptions'!$B$12+B39*'India Assumptions'!$B$13</f>
+        <v/>
+      </c>
+      <c r="C45" s="25">
+        <f>C38*'India Assumptions'!$B$12+C39*'India Assumptions'!$B$13</f>
+        <v/>
+      </c>
+      <c r="D45" s="25">
+        <f>D38*'India Assumptions'!$B$12+D39*'India Assumptions'!$B$13</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:F29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Unit Economics (India)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="14" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B3" s="9" t="inlineStr">
+        <is>
+          <t>SMB</t>
+        </is>
+      </c>
+      <c r="C3" s="9" t="inlineStr">
+        <is>
+          <t>Mid</t>
+        </is>
+      </c>
+      <c r="D3" s="9" t="inlineStr">
+        <is>
+          <t>Blended</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>weights</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>n</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>ACV / yr</t>
+        </is>
+      </c>
+      <c r="B4" s="25">
+        <f>'India Assumptions'!B10</f>
+        <v/>
+      </c>
+      <c r="C4" s="25">
+        <f>'India Assumptions'!B11</f>
+        <v/>
+      </c>
+      <c r="D4" s="24">
+        <f>(B4*$F$4+C4*$F$5)/($F$4+$F$5)</f>
+        <v/>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>SMB logos (Base)</t>
+        </is>
+      </c>
+      <c r="F4" s="15">
+        <f>SUM('India Assumptions'!B23:D23)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Sites per customer</t>
+        </is>
+      </c>
+      <c r="B5" s="11">
+        <f>'India Assumptions'!B42</f>
+        <v/>
+      </c>
+      <c r="C5" s="11">
+        <f>'India Assumptions'!B43</f>
+        <v/>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Mid logos (Base)</t>
+        </is>
+      </c>
+      <c r="F5" s="15">
+        <f>SUM('India Assumptions'!B24:D24)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>COGS — hosting &amp; infra</t>
+        </is>
+      </c>
+      <c r="B6" s="25">
+        <f>B5*'India Assumptions'!$B$36</f>
+        <v/>
+      </c>
+      <c r="C6" s="25">
+        <f>C5*'India Assumptions'!$B$36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>COGS — CAD-conversion compute</t>
+        </is>
+      </c>
+      <c r="B7" s="25">
+        <f>0</f>
+        <v/>
+      </c>
+      <c r="C7" s="25">
+        <f>C5*'India Assumptions'!$B$37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>COGS — support / CS</t>
+        </is>
+      </c>
+      <c r="B8" s="25">
+        <f>B5*'India Assumptions'!$B$38</f>
+        <v/>
+      </c>
+      <c r="C8" s="25">
+        <f>C5*'India Assumptions'!$B$38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>COGS — payments</t>
+        </is>
+      </c>
+      <c r="B9" s="25">
+        <f>B4*'India Assumptions'!$B$39</f>
+        <v/>
+      </c>
+      <c r="C9" s="25">
+        <f>C4*'India Assumptions'!$B$39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Total COGS</t>
+        </is>
+      </c>
+      <c r="B10" s="25">
+        <f>SUM(B6:B9)</f>
+        <v/>
+      </c>
+      <c r="C10" s="25">
+        <f>SUM(C6:C9)</f>
+        <v/>
+      </c>
+      <c r="D10" s="24">
+        <f>(B10*$F$4+C10*$F$5)/($F$4+$F$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Gross profit / yr</t>
+        </is>
+      </c>
+      <c r="B11" s="25">
+        <f>B4-B10</f>
+        <v/>
+      </c>
+      <c r="C11" s="25">
+        <f>C4-C10</f>
+        <v/>
+      </c>
+      <c r="D11" s="24">
+        <f>(B11*$F$4+C11*$F$5)/($F$4+$F$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="8" t="inlineStr">
+        <is>
+          <t>Gross margin %</t>
+        </is>
+      </c>
+      <c r="B12" s="16">
+        <f>B11/B4</f>
+        <v/>
+      </c>
+      <c r="C12" s="16">
+        <f>C11/C4</f>
+        <v/>
+      </c>
+      <c r="D12" s="17">
+        <f>D11/D4</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>CAC per logo</t>
+        </is>
+      </c>
+      <c r="B14" s="25">
+        <f>'India Assumptions'!B31</f>
+        <v/>
+      </c>
+      <c r="C14" s="25">
+        <f>'India Assumptions'!B32</f>
+        <v/>
+      </c>
+      <c r="D14" s="24">
+        <f>(B14*$F$4+C14*$F$5)/($F$4+$F$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Onboarding fee</t>
+        </is>
+      </c>
+      <c r="B15" s="25">
+        <f>'India Assumptions'!B12</f>
+        <v/>
+      </c>
+      <c r="C15" s="25">
+        <f>'India Assumptions'!B13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Onboarding gross profit</t>
+        </is>
+      </c>
+      <c r="B16" s="25">
+        <f>B15*'India Assumptions'!$B$33</f>
+        <v/>
+      </c>
+      <c r="C16" s="25">
+        <f>C15*'India Assumptions'!$B$33</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Net CAC (CAC − onb. GP)</t>
+        </is>
+      </c>
+      <c r="B17" s="25">
+        <f>B14-B16</f>
+        <v/>
+      </c>
+      <c r="C17" s="25">
+        <f>C14-C16</f>
+        <v/>
+      </c>
+      <c r="D17" s="24">
+        <f>(B17*$F$4+C17*$F$5)/($F$4+$F$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Monthly gross profit</t>
+        </is>
+      </c>
+      <c r="B19" s="25">
+        <f>B11/12</f>
+        <v/>
+      </c>
+      <c r="C19" s="25">
+        <f>C11/12</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>CAC payback (gross)</t>
+        </is>
+      </c>
+      <c r="B20" s="18">
+        <f>B14/B19</f>
+        <v/>
+      </c>
+      <c r="C20" s="18">
+        <f>C14/C19</f>
+        <v/>
+      </c>
+      <c r="D20" s="19">
+        <f>D14/(D11/12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="8" t="inlineStr">
+        <is>
+          <t>Net CAC payback</t>
+        </is>
+      </c>
+      <c r="B21" s="18">
+        <f>B17/B19</f>
+        <v/>
+      </c>
+      <c r="C21" s="18">
+        <f>C17/C19</f>
+        <v/>
+      </c>
+      <c r="D21" s="19">
+        <f>D17/(D11/12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Logo churn / yr</t>
+        </is>
+      </c>
+      <c r="B23" s="16">
+        <f>'India Assumptions'!B18</f>
+        <v/>
+      </c>
+      <c r="C23" s="16">
+        <f>'India Assumptions'!B19</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Customer lifetime (yrs)</t>
+        </is>
+      </c>
+      <c r="B24" s="20">
+        <f>1/B23</f>
+        <v/>
+      </c>
+      <c r="C24" s="20">
+        <f>1/C23</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>LTV (gross margin)</t>
+        </is>
+      </c>
+      <c r="B25" s="25">
+        <f>B11*B24</f>
+        <v/>
+      </c>
+      <c r="C25" s="25">
+        <f>C11*C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="24">
+        <f>(B25*$F$4+C25*$F$5)/($F$4+$F$5)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>LTV:CAC (gross)</t>
+        </is>
+      </c>
+      <c r="B26" s="21">
+        <f>B25/B14</f>
+        <v/>
+      </c>
+      <c r="C26" s="21">
+        <f>C25/C14</f>
+        <v/>
+      </c>
+      <c r="D26" s="22">
+        <f>D25/D14</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="8" t="inlineStr">
+        <is>
+          <t>LTV:CAC (net CAC)</t>
+        </is>
+      </c>
+      <c r="B27" s="21">
+        <f>B25/B17</f>
+        <v/>
+      </c>
+      <c r="C27" s="21">
+        <f>C25/C17</f>
+        <v/>
+      </c>
+      <c r="D27" s="22">
+        <f>D25/D17</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="27" t="inlineStr">
+        <is>
+          <t>Note: SMB excludes CAD compute (SMB = non-3D tiers). Mid = Digital Twin tier (CAD applies).</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>